<commit_message>
atualização das análises - e geração de PDF para não programadores
</commit_message>
<xml_diff>
--- a/R Markdown/dados/ivu_subprefeituras_2025.xlsx
+++ b/R Markdown/dados/ivu_subprefeituras_2025.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cloudprodamazhotmail-my.sharepoint.com/personal/gabrielmachado_prefeitura_sp_gov_br/Documents/Área de Trabalho/IDRGP/IDRGP 2025/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cloudprodamazhotmail-my.sharepoint.com/personal/gabrielmachado_prefeitura_sp_gov_br/Documents/Área de Trabalho/IDRGP/IDRGP-2025/R Markdown/dados/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="13" documentId="8_{E1B51FC3-EE73-4DD2-B1AB-F92D24E15DA2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EBB52D98-C8B3-4316-8241-5DC1879AC13F}"/>
+  <xr:revisionPtr revIDLastSave="20" documentId="8_{E1B51FC3-EE73-4DD2-B1AB-F92D24E15DA2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5630736F-6F75-4502-8BE4-2DEE73AB8E24}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="subprefeituras_dados" sheetId="1" r:id="rId1"/>
@@ -733,6 +733,13 @@
     <col min="6" max="6" width="16.85546875" customWidth="1"/>
     <col min="7" max="7" width="31.7109375" customWidth="1"/>
     <col min="8" max="8" width="31.85546875" customWidth="1"/>
+    <col min="9" max="9" width="33.85546875" customWidth="1"/>
+    <col min="10" max="10" width="33.140625" customWidth="1"/>
+    <col min="11" max="11" width="30.140625" customWidth="1"/>
+    <col min="12" max="12" width="42.140625" customWidth="1"/>
+    <col min="13" max="13" width="33.5703125" customWidth="1"/>
+    <col min="14" max="14" width="36" customWidth="1"/>
+    <col min="16" max="16" width="34" customWidth="1"/>
     <col min="17" max="17" width="26.28515625" customWidth="1"/>
     <col min="21" max="21" width="47.7109375" customWidth="1"/>
     <col min="25" max="25" width="18.28515625" customWidth="1"/>
@@ -3285,6 +3292,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100506FD4652602C740A483E9D3DF6A153B" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="3ae790dad332779219ad741447ce1449">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="1aa39b8c-19b3-4ca5-9ada-a1970df5e875" xmlns:ns3="a9968193-2d77-4b73-840a-26fc33ae728b" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="bceb73c01ba1e25437ffc1b7a59fee3b" ns2:_="" ns3:_="">
     <xsd:import namespace="1aa39b8c-19b3-4ca5-9ada-a1970df5e875"/>
@@ -3539,15 +3555,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -3560,6 +3567,14 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5075A89E-4FDE-447E-AC41-A26DF22DC565}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3BF825F9-0948-4560-8B2C-B62AF591D545}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -3578,14 +3593,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5075A89E-4FDE-447E-AC41-A26DF22DC565}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{69F5E1FC-361F-46D1-8C07-01719E84611F}">
   <ds:schemaRefs>
@@ -3595,4 +3602,10 @@
     <ds:schemaRef ds:uri="a9968193-2d77-4b73-840a-26fc33ae728b"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
+<clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
+  <clbl:label id="{f398df9c-fd0c-4829-a003-c770a1c4a063}" enabled="0" method="" siteId="{f398df9c-fd0c-4829-a003-c770a1c4a063}" removed="1"/>
+</clbl:labelList>
 </file>
</xml_diff>